<commit_message>
Added new pages to the framework
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/myTestData.xlsx
+++ b/src/test/resources/TestData/myTestData.xlsx
@@ -5,15 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mogaupavlovmalepe/Documents/My Apps/Pablo Automation Frameworks/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mogaupavlovmalepe/Documents/My Apps/Pablo Automation Frameworks/NdosiBootcamp_SelenuimJavaAssessment/src/test/resources/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0306581D-7787-734F-B4E6-892AFC2F2E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8449787E-6012-D040-B2C1-8C3F2E174C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="17260" xr2:uid="{84C3D3D2-A915-944C-A26C-C00D0E7AB408}"/>
+    <workbookView xWindow="9220" yWindow="2460" windowWidth="19800" windowHeight="7840" activeTab="2" xr2:uid="{84C3D3D2-A915-944C-A26C-C00D0E7AB408}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_Credentials" sheetId="1" r:id="rId1"/>
+    <sheet name="Order_Details" sheetId="2" r:id="rId2"/>
+    <sheet name="Order_Preview" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,19 +38,76 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Username</t>
   </si>
   <si>
     <t>Password</t>
+  </si>
+  <si>
+    <t>pablo@gmail.com</t>
+  </si>
+  <si>
+    <t>Pablo123!**</t>
+  </si>
+  <si>
+    <t>Device_Type</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>128GB</t>
+  </si>
+  <si>
+    <t>Deliver_Address</t>
+  </si>
+  <si>
+    <t>123 Test Street</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>ShippingMethod</t>
+  </si>
+  <si>
+    <t>Warranty</t>
+  </si>
+  <si>
+    <t>Discount_Code</t>
+  </si>
+  <si>
+    <t>Express (+R25)</t>
+  </si>
+  <si>
+    <t>1 Year (+R49)</t>
+  </si>
+  <si>
+    <t>SAVE10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -62,6 +121,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0F3D4A"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -84,9 +149,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,8 +487,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E32D5B1-862F-8046-8D9D-908EDC4339AC}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -430,6 +499,106 @@
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32825867-7A92-3747-B6F8-2121A1B45A03}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="14.1640625" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{500935D0-3F73-5943-8783-2F08BF50D769}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="23.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>